<commit_message>
deploy: 2026-07-07 19:41 (build 20260707194149)
</commit_message>
<xml_diff>
--- a/cloudflare-deploy/public/library/student/student-en.xlsx
+++ b/cloudflare-deploy/public/library/student/student-en.xlsx
@@ -1108,7 +1108,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>🌐 test.mangoi.co.kr    📞 1588-0000    ✉ support@mangoi.co.kr</t>
+          <t>🌐 www.mangoi.co.kr    📞 1644-0561    ✉ support@mangoi.co.kr</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Go to test.mangoi.co.kr in your browser and log in (social login works too). → Check your name and points (P) at the top-right to confirm you're logged in. → Tap the 'Open' tab on the left to expand the menu sidebar. → Ask the A.i assistant at the bottom-right anything you're curious about. → Use the EN button to switch the on-screen text to English.</t>
+          <t>Go to www.mangoi.co.kr in your browser and log in (social login works too). → Check your name and points (P) at the top-right to confirm you're logged in. → Tap the 'Open' tab on the left to expand the menu sidebar. → Ask the A.i assistant at the bottom-right anything you're curious about. → Use the EN button to switch the on-screen text to English.</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>Go to test.mangoi.co.kr in your browser and log in (social login works too).</t>
+          <t>Go to www.mangoi.co.kr in your browser and log in (social login works too).</t>
         </is>
       </c>
     </row>

</xml_diff>